<commit_message>
Some cod mapped that was failling and making wrong calculations are being corrected
</commit_message>
<xml_diff>
--- a/Map Opeperation/Relatorio_61_PARTEN.xlsx
+++ b/Map Opeperation/Relatorio_61_PARTEN.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perna\Desktop\STALLANTIS\Volume_Accuracy\Map Opeperation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB17A0F8-ECFE-4230-ADC2-FD110C67475E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BBC9FAEE-CF5C-4F03-9142-899A658F2AB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="35">
   <si>
     <t>excluded</t>
   </si>
@@ -115,13 +115,37 @@
   </si>
   <si>
     <t>MY(26)+,(029,097,392)+</t>
+  </si>
+  <si>
+    <t>FAASA</t>
+  </si>
+  <si>
+    <t>014+,025-</t>
+  </si>
+  <si>
+    <t>(0YF,400,JRC)-</t>
+  </si>
+  <si>
+    <t>(048,LPU)+</t>
+  </si>
+  <si>
+    <t>CCH+</t>
+  </si>
+  <si>
+    <t>(051,LNV)-</t>
+  </si>
+  <si>
+    <t>101+,(051,LNV)-</t>
+  </si>
+  <si>
+    <t>(0YF,400)+</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,8 +186,15 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -173,6 +204,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF002060"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9966"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -193,8 +230,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="1" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -204,8 +243,6 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -213,9 +250,13 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{A146EDCC-61B0-4BF3-BDEE-C2422EC0B4E6}"/>
+    <cellStyle name="Percent 2" xfId="2" xr:uid="{F2473930-727A-43EC-924F-6A1EADB84FCD}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -518,7 +559,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="4"/>
@@ -526,10 +567,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -537,102 +578,55 @@
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>3</v>
+      <c r="B2" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>20</v>
+        <v>9</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>8</v>
+        <v>27</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>21</v>
+      <c r="B5" s="8" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>22</v>
+      <c r="B6" s="8" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>13</v>
+      <c r="A7" s="2"/>
+      <c r="B7" s="8" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>15</v>
-      </c>
+      <c r="A8" s="2"/>
+      <c r="B8" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9"/>
     </row>
     <row r="10" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B12" s="7"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B13" s="7"/>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B14" s="7"/>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B15" s="7"/>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B16" s="7"/>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B17" s="7"/>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B18" s="6"/>
+      <c r="A10" s="2"/>
+      <c r="B10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -656,10 +650,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="7" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -676,7 +670,7 @@
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="4" t="s">
@@ -687,7 +681,7 @@
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -704,7 +698,7 @@
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -721,7 +715,7 @@
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -738,7 +732,7 @@
       <c r="A6" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
@@ -749,7 +743,7 @@
       <c r="A7" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="4" t="s">
@@ -760,7 +754,7 @@
       <c r="A8" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -777,7 +771,7 @@
       <c r="A9" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -791,36 +785,36 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="2" t="s">
         <v>6</v>
       </c>
     </row>
@@ -834,8 +828,274 @@
 </worksheet>
 </file>
 
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="e13b492c-44e0-478c-a27b-4b735264ccb7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1096d648-6e9c-4990-8f73-aa0f2ab1a217">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CA1DFDF4B147C34BB45DD9C94654ACC2" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="897bd39cf1d1b4d81f36a51d3a3e06a6">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1096d648-6e9c-4990-8f73-aa0f2ab1a217" xmlns:ns3="e13b492c-44e0-478c-a27b-4b735264ccb7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6707c27936323c15de64aa66c05905b8" ns2:_="" ns3:_="">
+    <xsd:import namespace="1096d648-6e9c-4990-8f73-aa0f2ab1a217"/>
+    <xsd:import namespace="e13b492c-44e0-478c-a27b-4b735264ccb7"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="1096d648-6e9c-4990-8f73-aa0f2ab1a217" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="14" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="9247bebf-ce0e-4fa1-bae7-748a1283d6fa" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="18" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="19" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:description="" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e13b492c-44e0-478c-a27b-4b735264ccb7" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="17" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{a993a088-c5ed-4b9a-9cf0-e9a75d274e9d}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e13b492c-44e0-478c-a27b-4b735264ccb7">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A053CB02-5652-4784-A7C4-82E07D67290C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8291598-7014-41C0-BCA7-DED85A1D138E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e13b492c-44e0-478c-a27b-4b735264ccb7"/>
+    <ds:schemaRef ds:uri="1096d648-6e9c-4990-8f73-aa0f2ab1a217"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1875EB00-CEAB-4752-8DCA-10AF49A43271}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1096d648-6e9c-4990-8f73-aa0f2ab1a217"/>
+    <ds:schemaRef ds:uri="e13b492c-44e0-478c-a27b-4b735264ccb7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{4cde0bb8-21e0-4ae3-9906-7ac25165b779}" enabled="1" method="Privileged" siteId="{d852d5cd-724c-4128-8812-ffa5db3f8507}" contentBits="0" removed="0"/>
   <clbl:label id="{736915f3-2f02-4945-8997-f2963298db46}" enabled="1" method="Standard" siteId="{cd99fef8-1cd3-4a2a-9bdf-15531181d65e}" contentBits="1" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>